<commit_message>
substituted backordered components and created assembly guide
</commit_message>
<xml_diff>
--- a/orderlist.xlsx
+++ b/orderlist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order list" sheetId="1" r:id="Rcca39aa414c04597"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order list" sheetId="1" r:id="R85a3d17ec2804c29"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -439,7 +439,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="str">
-        <v>120 fitted components. Order 129 pieces across 21 purchase lines.</v>
+        <v>120 fitted components. Order 144 pieces across 21 purchase lines.</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -458,7 +458,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="str">
-        <v>2026-10-29 listing snapshots. USD excludes shipping, tax and tariffs. Standardized CAD; circuit connectivity unchanged.</v>
+        <v>Stock/prices: 2026-10-29; 10k/100k replacements checked 2026-10-30. USD excludes shipping, tax and tariffs.</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -545,14 +545,14 @@
         <v>8</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="19" t="n">
         <v>2.3</v>
       </c>
       <c r="E7" s="20" t="n">
         <f>ROUND(C7*D7,2)</f>
-        <v>18.4</v>
+        <v>20.7</v>
       </c>
       <c r="F7" s="22" t="n">
         <v>1218</v>
@@ -562,7 +562,7 @@
       </c>
       <c r="H7" s="20" t="n">
         <f>ROUND(C7*G7,2)</f>
-        <v>18.4</v>
+        <v>20.7</v>
       </c>
       <c r="I7" s="22" t="n">
         <v>6897</v>
@@ -580,7 +580,9 @@
       <c r="N7" s="14" t="str">
         <v>BreakoutBoard:SSOP-28_5.3x10.2mm_P0.65mm</v>
       </c>
-      <c r="O7" s="14" t="str"/>
+      <c r="O7" s="14" t="str">
+        <v>8 fitted; 1 spare(s).</v>
+      </c>
     </row>
     <row r="8" ht="25" customHeight="1">
       <c r="A8" s="25" t="str">
@@ -590,14 +592,14 @@
         <v>8</v>
       </c>
       <c r="C8" s="26" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="27" t="n">
         <v>0.62</v>
       </c>
       <c r="E8" s="28" t="n">
         <f>ROUND(C8*D8,2)</f>
-        <v>4.96</v>
+        <v>5.58</v>
       </c>
       <c r="F8" s="29" t="n">
         <v>389</v>
@@ -607,7 +609,7 @@
       </c>
       <c r="H8" s="28" t="n">
         <f>ROUND(C8*G8,2)</f>
-        <v>4.96</v>
+        <v>5.58</v>
       </c>
       <c r="I8" s="29" t="n">
         <v>1362</v>
@@ -625,7 +627,9 @@
       <c r="N8" s="14" t="str">
         <v>BreakoutBoard:Crystal_SMD_Abracon_ABM8G-4Pin_3.2x2.5mm</v>
       </c>
-      <c r="O8" s="14" t="str"/>
+      <c r="O8" s="14" t="str">
+        <v>8 fitted; 1 spare(s).</v>
+      </c>
     </row>
     <row r="9" ht="25" customHeight="1">
       <c r="A9" s="14" t="str">
@@ -635,14 +639,14 @@
         <v>1</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="19" t="n">
         <v>0.45</v>
       </c>
       <c r="E9" s="20" t="n">
         <f>ROUND(C9*D9,2)</f>
-        <v>0.45</v>
+        <v>0.9</v>
       </c>
       <c r="F9" s="22" t="n">
         <v>82294</v>
@@ -652,7 +656,7 @@
       </c>
       <c r="H9" s="20" t="n">
         <f>ROUND(C9*G9,2)</f>
-        <v>0.44</v>
+        <v>0.88</v>
       </c>
       <c r="I9" s="22" t="n">
         <v>49482</v>
@@ -670,7 +674,9 @@
       <c r="N9" s="14" t="str">
         <v>BreakoutBoard:SOT-23-5</v>
       </c>
-      <c r="O9" s="14" t="str"/>
+      <c r="O9" s="14" t="str">
+        <v>1 fitted; 1 spare(s).</v>
+      </c>
     </row>
     <row r="10" ht="25" customHeight="1">
       <c r="A10" s="25" t="str">
@@ -680,14 +686,14 @@
         <v>16</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D10" s="27" t="n">
         <v>0.028</v>
       </c>
       <c r="E10" s="28" t="n">
         <f>ROUND(C10*D10,2)</f>
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="F10" s="29" t="n">
         <v>1471</v>
@@ -716,7 +722,7 @@
         <v>Capacitor_SMD:C_0603_1608Metric</v>
       </c>
       <c r="O10" s="14" t="str">
-        <v>Exact listing found; stock and USD price not verified. Buy the specified Samsung part from DigiKey.</v>
+        <v>16 fitted; 2 spare(s).</v>
       </c>
     </row>
     <row r="11" ht="25" customHeight="1">
@@ -727,14 +733,14 @@
         <v>28</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D11" s="19" t="n">
         <v>0.08</v>
       </c>
       <c r="E11" s="20" t="n">
         <f>ROUND(C11*D11,2)</f>
-        <v>2.24</v>
+        <v>2.4</v>
       </c>
       <c r="F11" s="22" t="n">
         <v>62814</v>
@@ -744,7 +750,7 @@
       </c>
       <c r="H11" s="20" t="n">
         <f>ROUND(C11*G11,2)</f>
-        <v>2.04</v>
+        <v>2.19</v>
       </c>
       <c r="I11" s="22" t="n">
         <v>47009219</v>
@@ -763,7 +769,7 @@
         <v>BreakoutBoard:C_0603_1608Metric</v>
       </c>
       <c r="O11" s="14" t="str">
-        <v>28 x 100 nF bypass capacitors: C1 and C21-C47. MPN retained in hidden fields.</v>
+        <v>28 x 100 nF bypass capacitors: C1 and C21-C47. MPN retained in hidden fields. 28 fitted; 2 spare(s).</v>
       </c>
     </row>
     <row r="12" ht="25" customHeight="1">
@@ -774,14 +780,14 @@
         <v>2</v>
       </c>
       <c r="C12" s="26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="27" t="n">
         <v>0.17</v>
       </c>
       <c r="E12" s="28" t="n">
         <f>ROUND(C12*D12,2)</f>
-        <v>0.34</v>
+        <v>0.51</v>
       </c>
       <c r="F12" s="29" t="n">
         <v>1368662</v>
@@ -791,7 +797,7 @@
       </c>
       <c r="H12" s="28" t="n">
         <f>ROUND(C12*G12,2)</f>
-        <v>0.34</v>
+        <v>0.51</v>
       </c>
       <c r="I12" s="29" t="n">
         <v>1426652</v>
@@ -810,7 +816,7 @@
         <v>BreakoutBoard:C_0603_1608Metric</v>
       </c>
       <c r="O12" s="14" t="str">
-        <v>Stock and USD pricing from Mouser US category listing.</v>
+        <v>2 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="13" ht="25" customHeight="1">
@@ -821,14 +827,14 @@
         <v>1</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="19" t="n">
         <v>0.27</v>
       </c>
       <c r="E13" s="20" t="n">
         <f>ROUND(C13*D13,2)</f>
-        <v>0.27</v>
+        <v>0.54</v>
       </c>
       <c r="F13" s="22" t="n">
         <v>187206</v>
@@ -838,7 +844,7 @@
       </c>
       <c r="H13" s="20" t="n">
         <f>ROUND(C13*G13,2)</f>
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I13" s="22" t="str">
         <v>Unverified</v>
@@ -857,7 +863,7 @@
         <v>BreakoutBoard:C_0805_2012Metric</v>
       </c>
       <c r="O13" s="14" t="str">
-        <v>Exact E suffix. USD price from Mouser Israel; current stock not verified. Do not replace with the G suffix automatically.</v>
+        <v>1 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="14" ht="25" customHeight="1">
@@ -868,24 +874,24 @@
         <v>8</v>
       </c>
       <c r="C14" s="26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="27" t="n">
-        <v>0.047</v>
+        <v>0.1</v>
       </c>
       <c r="E14" s="28" t="n">
         <f>ROUND(C14*D14,2)</f>
-        <v>0.47</v>
+        <v>0.9</v>
       </c>
       <c r="F14" s="29" t="n">
         <v>131576</v>
       </c>
       <c r="G14" s="27" t="n">
-        <v>0.025</v>
+        <v>0.1</v>
       </c>
       <c r="H14" s="28" t="n">
         <f>ROUND(C14*G14,2)</f>
-        <v>0.25</v>
+        <v>0.9</v>
       </c>
       <c r="I14" s="29" t="n">
         <v>120281</v>
@@ -904,12 +910,12 @@
         <v>BreakoutBoard:R_1206_3216Metric</v>
       </c>
       <c r="O14" s="14" t="str">
-        <v>All eight CAN termination resistors use this 1206, 120-ohm, 1%, 0.25 W part. Order 10 instead of 8: the quantity discount lowers the line total.</v>
+        <v>All eight CAN termination resistors use this 1206, 120-ohm, 1%, 0.25 W part. 8 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="15" ht="25" customHeight="1">
       <c r="A15" s="14" t="str">
-        <v>RC0603FR-0710KL</v>
+        <v>AC0603FR-0710KL</v>
       </c>
       <c r="B15" s="17" t="n">
         <v>9</v>
@@ -918,24 +924,24 @@
         <v>10</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="E15" s="20" t="n">
         <f>ROUND(C15*D15,2)</f>
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="F15" s="22" t="n">
-        <v>2396093</v>
-      </c>
-      <c r="G15" s="19" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="H15" s="20" t="n">
-        <f>ROUND(C15*G15,2)</f>
-        <v>0.14</v>
-      </c>
-      <c r="I15" s="22" t="n">
-        <v>2782034</v>
+        <v>971121</v>
+      </c>
+      <c r="G15" s="19" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="H15" s="20" t="str">
+        <f>"n.a."</f>
+        <v>n.a.</v>
+      </c>
+      <c r="I15" s="22" t="str">
+        <v>Unverified</v>
       </c>
       <c r="J15" s="24" t="str">
         <v>DigiKey</v>
@@ -951,38 +957,38 @@
         <v>BreakoutBoard:R_0603_1608Metric</v>
       </c>
       <c r="O15" s="14" t="str">
-        <v>Order 10 instead of 9: the quantity discount lowers the line total.</v>
+        <v>CAD MPN: RC0603FR-0710KL. Original RC0603FR-0710KL is out of stock at DigiKey. AC0603FR-0710KL matches its resistance, tolerance, power, TCR and 1.60 x 0.80 x 0.45 mm nominal body. Purchase this compatible substitute for the existing 0603 footprint; no CAD or Gerber changes. 9 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="25" t="str">
-        <v>RC0603FR-07100KL</v>
+        <v>CRCW0603100KFKEA</v>
       </c>
       <c r="B16" s="26" t="n">
         <v>4</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>0.025</v>
+        <v>0.1</v>
       </c>
       <c r="E16" s="28" t="n">
         <f>ROUND(C16*D16,2)</f>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>2081432</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="H16" s="28" t="n">
-        <f>ROUND(C16*G16,2)</f>
-        <v>0.14</v>
-      </c>
-      <c r="I16" s="29" t="n">
-        <v>4585377</v>
+        <v>3055789</v>
+      </c>
+      <c r="G16" s="27" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="H16" s="28" t="str">
+        <f>"n.a."</f>
+        <v>n.a.</v>
+      </c>
+      <c r="I16" s="29" t="str">
+        <v>Unverified</v>
       </c>
       <c r="J16" s="30" t="str">
         <v>DigiKey</v>
@@ -998,7 +1004,7 @@
         <v>BreakoutBoard:R_0603_1608Metric</v>
       </c>
       <c r="O16" s="14" t="str">
-        <v>Order 10 instead of 4: the quantity discount lowers the line total.</v>
+        <v>CAD MPN: RC0603FR-07100KL. Original RC0603FR-07100KL is on backorder at DigiKey. CRCW0603100KFKEA matches 100 kohm, 1%, at least 0.1 W and 100 ppm/C. Its standard 0603 body (nominal 1.55 x 0.85 x 0.45 mm) fits the existing IPC-7351 nominal R_0603_1608Metric footprint. The manufacturer specifies 0.10 W standard / 0.125 W extended operation. No schematic, PCB or Gerber change is required. 4 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="17" ht="25" customHeight="1">
@@ -1009,14 +1015,14 @@
         <v>16</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D17" s="19" t="n">
         <v>0.025</v>
       </c>
       <c r="E17" s="20" t="n">
         <f>ROUND(C17*D17,2)</f>
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="F17" s="22" t="n">
         <v>1088640</v>
@@ -1026,7 +1032,7 @@
       </c>
       <c r="H17" s="20" t="n">
         <f>ROUND(C17*G17,2)</f>
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="I17" s="22" t="n">
         <v>595649</v>
@@ -1044,7 +1050,9 @@
       <c r="N17" s="14" t="str">
         <v>BreakoutBoard:R_0603_1608Metric</v>
       </c>
-      <c r="O17" s="14" t="str"/>
+      <c r="O17" s="14" t="str">
+        <v>16 fitted; 2 spare(s).</v>
+      </c>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="A18" s="25" t="str">
@@ -1054,14 +1062,14 @@
         <v>8</v>
       </c>
       <c r="C18" s="26" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D18" s="27" t="n">
         <v>0.13</v>
       </c>
       <c r="E18" s="28" t="n">
         <f>ROUND(C18*D18,2)</f>
-        <v>1.04</v>
+        <v>1.17</v>
       </c>
       <c r="F18" s="29" t="n">
         <v>120351</v>
@@ -1071,7 +1079,7 @@
       </c>
       <c r="H18" s="28" t="n">
         <f>ROUND(C18*G18,2)</f>
-        <v>1.04</v>
+        <v>1.17</v>
       </c>
       <c r="I18" s="29" t="str">
         <v>Unverified</v>
@@ -1090,7 +1098,7 @@
         <v>BreakoutBoard:JST_XH_B3B-XH-A_1x03_P2.50mm_Vertical</v>
       </c>
       <c r="O18" s="14" t="str">
-        <v>Listing uses B3B-XH-A(LF)(SN). Stock not verified. No black, reverse, or press-fit variants selected.</v>
+        <v>8 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="19" ht="25" customHeight="1">
@@ -1101,14 +1109,14 @@
         <v>1</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="19" t="n">
         <v>0.1</v>
       </c>
       <c r="E19" s="20" t="n">
         <f>ROUND(C19*D19,2)</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="F19" s="22" t="n">
         <v>320857</v>
@@ -1118,7 +1126,7 @@
       </c>
       <c r="H19" s="20" t="n">
         <f>ROUND(C19*G19,2)</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I19" s="22" t="n">
         <v>560</v>
@@ -1137,7 +1145,7 @@
         <v>BreakoutBoard:JST_XH_B2B-XH-A_1x02_P2.50mm_Vertical</v>
       </c>
       <c r="O19" s="14" t="str">
-        <v>Listing uses B2B-XH-A(LF)(SN). Stock evidence from Mouser South Africa. No A-M/press-fit variant selected.</v>
+        <v>1 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1">
@@ -1148,14 +1156,14 @@
         <v>1</v>
       </c>
       <c r="C20" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="27" t="n">
         <v>4.34</v>
       </c>
       <c r="E20" s="28" t="n">
         <f>ROUND(C20*D20,2)</f>
-        <v>4.34</v>
+        <v>8.68</v>
       </c>
       <c r="F20" s="29" t="n">
         <v>4597</v>
@@ -1165,7 +1173,7 @@
       </c>
       <c r="H20" s="28" t="n">
         <f>ROUND(C20*G20,2)</f>
-        <v>4.13</v>
+        <v>8.26</v>
       </c>
       <c r="I20" s="29" t="n">
         <v>1973</v>
@@ -1184,7 +1192,7 @@
         <v>Connector_PinSocket_2.54mm:PinSocket_2x20_P2.54mm_Vertical</v>
       </c>
       <c r="O20" s="14" t="str">
-        <v>J1 consistently uses M20-7832046 and the female socket footprint in the schematic, PCB and order list.</v>
+        <v>J1 consistently uses M20-7832046 and the female socket footprint in the schematic, PCB and order list. 1 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="21" ht="25" customHeight="1">
@@ -1195,14 +1203,14 @@
         <v>1</v>
       </c>
       <c r="C21" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="19" t="n">
         <v>1.25</v>
       </c>
       <c r="E21" s="20" t="n">
         <f>ROUND(C21*D21,2)</f>
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="F21" s="22" t="n">
         <v>36548</v>
@@ -1212,7 +1220,7 @@
       </c>
       <c r="H21" s="20" t="n">
         <f>ROUND(C21*G21,2)</f>
-        <v>0.78</v>
+        <v>1.56</v>
       </c>
       <c r="I21" s="22" t="n">
         <v>45577</v>
@@ -1231,7 +1239,7 @@
         <v>BreakoutBoard:Fuse_1206_3216Metric</v>
       </c>
       <c r="O21" s="14" t="str">
-        <v>F1 is fitted in the current schematic and layout.</v>
+        <v>F1 is fitted in the current schematic and layout. 1 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="22" ht="25" customHeight="1">
@@ -1242,14 +1250,14 @@
         <v>1</v>
       </c>
       <c r="C22" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="27" t="n">
         <v>0.52</v>
       </c>
       <c r="E22" s="28" t="n">
         <f>ROUND(C22*D22,2)</f>
-        <v>0.52</v>
+        <v>1.04</v>
       </c>
       <c r="F22" s="29" t="n">
         <v>443245</v>
@@ -1278,7 +1286,7 @@
         <v>BreakoutBoard:SOT-23</v>
       </c>
       <c r="O22" s="14" t="str">
-        <v>Keep Alpha &amp; Omega AO3401A. No alternate MOSFET selected.</v>
+        <v>Keep Alpha &amp; Omega AO3401A. No alternate MOSFET selected. 1 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="23" ht="25" customHeight="1">
@@ -1289,14 +1297,14 @@
         <v>1</v>
       </c>
       <c r="C23" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="19" t="n">
         <v>0.22</v>
       </c>
       <c r="E23" s="20" t="n">
         <f>ROUND(C23*D23,2)</f>
-        <v>0.22</v>
+        <v>0.44</v>
       </c>
       <c r="F23" s="22" t="n">
         <v>6702</v>
@@ -1306,7 +1314,7 @@
       </c>
       <c r="H23" s="20" t="n">
         <f>ROUND(C23*G23,2)</f>
-        <v>0.21</v>
+        <v>0.42</v>
       </c>
       <c r="I23" s="22" t="n">
         <v>9830</v>
@@ -1324,7 +1332,9 @@
       <c r="N23" s="14" t="str">
         <v>BreakoutBoard:D_SOD-123</v>
       </c>
-      <c r="O23" s="14" t="str"/>
+      <c r="O23" s="14" t="str">
+        <v>1 fitted; 1 spare(s).</v>
+      </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="25" t="str">
@@ -1334,14 +1344,14 @@
         <v>1</v>
       </c>
       <c r="C24" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="27" t="n">
         <v>0.39</v>
       </c>
       <c r="E24" s="28" t="n">
         <f>ROUND(C24*D24,2)</f>
-        <v>0.39</v>
+        <v>0.78</v>
       </c>
       <c r="F24" s="29" t="n">
         <v>6890</v>
@@ -1351,7 +1361,7 @@
       </c>
       <c r="H24" s="28" t="n">
         <f>ROUND(C24*G24,2)</f>
-        <v>0.39</v>
+        <v>0.78</v>
       </c>
       <c r="I24" s="29" t="n">
         <v>3795</v>
@@ -1369,7 +1379,9 @@
       <c r="N24" s="14" t="str">
         <v>BreakoutBoard:TSSOP-14_4.4x5mm_P0.65mm</v>
       </c>
-      <c r="O24" s="14" t="str"/>
+      <c r="O24" s="14" t="str">
+        <v>1 fitted; 1 spare(s).</v>
+      </c>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="14" t="str">
@@ -1379,14 +1391,14 @@
         <v>2</v>
       </c>
       <c r="C25" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" s="19" t="n">
         <v>0.25</v>
       </c>
       <c r="E25" s="20" t="n">
         <f>ROUND(C25*D25,2)</f>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="F25" s="22" t="n">
         <v>6192</v>
@@ -1396,7 +1408,7 @@
       </c>
       <c r="H25" s="20" t="n">
         <f>ROUND(C25*G25,2)</f>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I25" s="22" t="n">
         <v>3867</v>
@@ -1414,7 +1426,9 @@
       <c r="N25" s="14" t="str">
         <v>BreakoutBoard:TSSOP-14_4.4x5mm_P0.65mm</v>
       </c>
-      <c r="O25" s="14" t="str"/>
+      <c r="O25" s="14" t="str">
+        <v>2 fitted; 1 spare(s).</v>
+      </c>
     </row>
     <row r="26" ht="25" customHeight="1">
       <c r="A26" s="25" t="str">
@@ -1424,14 +1438,14 @@
         <v>1</v>
       </c>
       <c r="C26" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="27" t="n">
         <v>0.32</v>
       </c>
       <c r="E26" s="28" t="n">
         <f>ROUND(C26*D26,2)</f>
-        <v>0.32</v>
+        <v>0.64</v>
       </c>
       <c r="F26" s="29" t="n">
         <v>4004</v>
@@ -1441,7 +1455,7 @@
       </c>
       <c r="H26" s="28" t="n">
         <f>ROUND(C26*G26,2)</f>
-        <v>0.28</v>
+        <v>0.56</v>
       </c>
       <c r="I26" s="29" t="n">
         <v>2760</v>
@@ -1459,7 +1473,9 @@
       <c r="N26" s="14" t="str">
         <v>BreakoutBoard:TSSOP-14_4.4x5mm_P0.65mm</v>
       </c>
-      <c r="O26" s="14" t="str"/>
+      <c r="O26" s="14" t="str">
+        <v>1 fitted; 1 spare(s).</v>
+      </c>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="14" t="str">
@@ -1469,14 +1485,14 @@
         <v>2</v>
       </c>
       <c r="C27" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27" s="19" t="n">
         <v>0.1</v>
       </c>
       <c r="E27" s="20" t="n">
         <f>ROUND(C27*D27,2)</f>
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="F27" s="22" t="n">
         <v>179951</v>
@@ -1486,7 +1502,7 @@
       </c>
       <c r="H27" s="20" t="n">
         <f>ROUND(C27*G27,2)</f>
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I27" s="22" t="n">
         <v>98136</v>
@@ -1505,7 +1521,7 @@
         <v>Connector_PinHeader_2.54mm:PinHeader_1x02_P2.54mm_Vertical</v>
       </c>
       <c r="O27" s="14" t="str">
-        <v>Fitted headers for TP13 and TP14. The other 21 test points are bare PCB pads.</v>
+        <v>Fitted headers for TP13 and TP14. The other 21 test points are bare PCB pads. 2 fitted; 1 spare(s).</v>
       </c>
     </row>
     <row r="28">
@@ -1535,12 +1551,12 @@
       </c>
       <c r="C29" s="36" t="n">
         <f>SUM(C7:C27)</f>
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="D29" s="37"/>
       <c r="E29" s="38" t="n">
         <f>SUM(E7:E27)</f>
-        <v>37.36</v>
+        <v>49.78</v>
       </c>
       <c r="F29" s="37"/>
       <c r="G29" s="37" t="str">
@@ -1576,7 +1592,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="str">
-        <v>Extras: 2 x 1206 120-ohm, 1 x 10-kohm, 6 x 100-kohm resistors. Published quantity breaks lower the line totals.</v>
+        <v>24 spare pieces: 20% extra overall, including at least one spare of every part type. Quantities match the bulk-add text.</v>
       </c>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1595,7 +1611,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="str">
-        <v>All eight terminations: RC1206FR-07120RL, 1206, 0.25 W. J1: M20-7832046 female socket. MPN fields match CAD.</v>
+        <v>Replacements: 10k AC0603FR-0710KL; 100k CRCW0603100KFKEA. Both fit existing 0603 footprints. CAD and Gerbers unchanged.</v>
       </c>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>

</xml_diff>